<commit_message>
Replace home page countdown offer with Winter Wonderland intro
The source home page swapped the time-limited "Book for 2027" countdown
teaser for a text intro (h1 title + h3 sub-heading, copy and arrow link).

- Import: map the "Page intro" section to the new h1 text teaser
  (handled by the existing columns-intro parser), keeping the
  countdown selector for when an offer returns; drop the grey style
- columns-intro: style the h1 title and h3 sub-heading used by the
  page intro, values taken from centerparcs.co.uk

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-home.report.xlsx
+++ b/tools/importer/reports/import-home.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>_reportFile</t>
   </si>
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero-notification","columns-offer","hero-video","tabs-village","carousel-lodges","columns-intro","columns-intro","columns-intro","cards-expand","cards-feature","cards-feature","carousel-activity","columns-promo","accordion-faq","accordion-faq"]</t>
+    <t>["hero-notification","hero-video","tabs-village","carousel-lodges","columns-intro","columns-intro","columns-intro","columns-intro","cards-expand","cards-feature","cards-feature","carousel-activity","columns-promo","accordion-faq","accordion-faq"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,13 +52,34 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-10-08T13:59:04.655Z</t>
+    <t>2026-10-14T13:03:03.451Z</t>
   </si>
   <si>
     <t>UK short breaks, designed to bring families together | Center Parcs</t>
   </si>
   <si>
     <t>https://www.centerparcs.co.uk/</t>
+  </si>
+  <si>
+    <t>discover-center-parcs/activities/outdoor-activities.report.json</t>
+  </si>
+  <si>
+    <t>["columns-intro","columns-intro","columns-intro","hero-video","cards-feature","cards-feature","cards-feature","carousel-activity","columns-promo","carousel-spotlight"]</t>
+  </si>
+  <si>
+    <t>discover-center-parcs/activities/outdoor-activities</t>
+  </si>
+  <si>
+    <t>activities</t>
+  </si>
+  <si>
+    <t>2026-10-12T09:33:55.752Z</t>
+  </si>
+  <si>
+    <t>Outdoor Activities | Center Parcs</t>
+  </si>
+  <si>
+    <t>https://www.centerparcs.co.uk/discover-center-parcs/activities/outdoor-activities.html</t>
   </si>
 </sst>
 </file>
@@ -447,16 +468,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="7" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="1" max="3" width="50" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="32" customWidth="1"/>
+    <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -509,6 +527,32 @@
       </c>
       <c r="H2" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>